<commit_message>
Fix toan bo chuc nang nhap xuat Excel
</commit_message>
<xml_diff>
--- a/backend/nhap_excel/mau_excel/mau_nhap_bo_mon.xlsx
+++ b/backend/nhap_excel/mau_excel/mau_nhap_bo_mon.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dữ liệu" sheetId="1" r:id="R82afc703f97b4cbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ví dụ" sheetId="2" r:id="Rb4550fb53aa64dde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="3" r:id="R243b9406f4e9441f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục" sheetId="4" r:id="Rbb210e70878043ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hệ thống" sheetId="5" r:id="R8a3f8d0b3e134032"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dữ liệu" sheetId="1" r:id="R651aac0eb6854ef4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ví dụ" sheetId="2" r:id="Rfc4cd070d4264729"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="3" r:id="Rc6a959fca98141c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh mục" sheetId="4" r:id="R7f679e91b2854fdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hệ thống" sheetId="5" r:id="Rc69be0f7feab47a9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,6 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="@"/>
+  </x:numFmts>
   <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
@@ -110,7 +113,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="55">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -211,6 +214,17 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -415,457 +429,462 @@
       <x:c r="A4" s="33" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B4" s="29" t="str"/>
-      <x:c r="C4" s="29" t="str"/>
-      <x:c r="D4" s="29" t="str"/>
-      <x:c r="E4" s="29" t="str"/>
+      <x:c r="B4" s="51" t="str"/>
+      <x:c r="C4" s="51" t="str"/>
+      <x:c r="D4" s="51" t="str"/>
+      <x:c r="E4" s="51" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="33" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B5" s="29" t="str"/>
-      <x:c r="C5" s="29" t="str"/>
-      <x:c r="D5" s="29" t="str"/>
-      <x:c r="E5" s="29" t="str"/>
+      <x:c r="B5" s="51" t="str"/>
+      <x:c r="C5" s="51" t="str"/>
+      <x:c r="D5" s="51" t="str"/>
+      <x:c r="E5" s="51" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="33" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B6" s="29" t="str"/>
-      <x:c r="C6" s="29" t="str"/>
-      <x:c r="D6" s="29" t="str"/>
-      <x:c r="E6" s="29" t="str"/>
+      <x:c r="B6" s="51" t="str"/>
+      <x:c r="C6" s="51" t="str"/>
+      <x:c r="D6" s="51" t="str"/>
+      <x:c r="E6" s="51" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="33" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B7" s="29" t="str"/>
-      <x:c r="C7" s="29" t="str"/>
-      <x:c r="D7" s="29" t="str"/>
-      <x:c r="E7" s="29" t="str"/>
+      <x:c r="B7" s="51" t="str"/>
+      <x:c r="C7" s="51" t="str"/>
+      <x:c r="D7" s="51" t="str"/>
+      <x:c r="E7" s="51" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="33" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B8" s="29" t="str"/>
-      <x:c r="C8" s="29" t="str"/>
-      <x:c r="D8" s="29" t="str"/>
-      <x:c r="E8" s="29" t="str"/>
+      <x:c r="B8" s="51" t="str"/>
+      <x:c r="C8" s="51" t="str"/>
+      <x:c r="D8" s="51" t="str"/>
+      <x:c r="E8" s="51" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="33" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B9" s="29" t="str"/>
-      <x:c r="C9" s="29" t="str"/>
-      <x:c r="D9" s="29" t="str"/>
-      <x:c r="E9" s="29" t="str"/>
+      <x:c r="B9" s="51" t="str"/>
+      <x:c r="C9" s="51" t="str"/>
+      <x:c r="D9" s="51" t="str"/>
+      <x:c r="E9" s="51" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="33" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B10" s="29" t="str"/>
-      <x:c r="C10" s="29" t="str"/>
-      <x:c r="D10" s="29" t="str"/>
-      <x:c r="E10" s="29" t="str"/>
+      <x:c r="B10" s="51" t="str"/>
+      <x:c r="C10" s="51" t="str"/>
+      <x:c r="D10" s="51" t="str"/>
+      <x:c r="E10" s="51" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="33" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B11" s="29" t="str"/>
-      <x:c r="C11" s="29" t="str"/>
-      <x:c r="D11" s="29" t="str"/>
-      <x:c r="E11" s="29" t="str"/>
+      <x:c r="B11" s="51" t="str"/>
+      <x:c r="C11" s="51" t="str"/>
+      <x:c r="D11" s="51" t="str"/>
+      <x:c r="E11" s="51" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="33" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B12" s="29" t="str"/>
-      <x:c r="C12" s="29" t="str"/>
-      <x:c r="D12" s="29" t="str"/>
-      <x:c r="E12" s="29" t="str"/>
+      <x:c r="B12" s="51" t="str"/>
+      <x:c r="C12" s="51" t="str"/>
+      <x:c r="D12" s="51" t="str"/>
+      <x:c r="E12" s="51" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="33" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B13" s="29" t="str"/>
-      <x:c r="C13" s="29" t="str"/>
-      <x:c r="D13" s="29" t="str"/>
-      <x:c r="E13" s="29" t="str"/>
+      <x:c r="B13" s="51" t="str"/>
+      <x:c r="C13" s="51" t="str"/>
+      <x:c r="D13" s="51" t="str"/>
+      <x:c r="E13" s="51" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="33" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B14" s="29" t="str"/>
-      <x:c r="C14" s="29" t="str"/>
-      <x:c r="D14" s="29" t="str"/>
-      <x:c r="E14" s="29" t="str"/>
+      <x:c r="B14" s="51" t="str"/>
+      <x:c r="C14" s="51" t="str"/>
+      <x:c r="D14" s="51" t="str"/>
+      <x:c r="E14" s="51" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="33" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B15" s="29" t="str"/>
-      <x:c r="C15" s="29" t="str"/>
-      <x:c r="D15" s="29" t="str"/>
-      <x:c r="E15" s="29" t="str"/>
+      <x:c r="B15" s="51" t="str"/>
+      <x:c r="C15" s="51" t="str"/>
+      <x:c r="D15" s="51" t="str"/>
+      <x:c r="E15" s="51" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="33" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B16" s="29" t="str"/>
-      <x:c r="C16" s="29" t="str"/>
-      <x:c r="D16" s="29" t="str"/>
-      <x:c r="E16" s="29" t="str"/>
+      <x:c r="B16" s="51" t="str"/>
+      <x:c r="C16" s="51" t="str"/>
+      <x:c r="D16" s="51" t="str"/>
+      <x:c r="E16" s="51" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="33" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B17" s="29" t="str"/>
-      <x:c r="C17" s="29" t="str"/>
-      <x:c r="D17" s="29" t="str"/>
-      <x:c r="E17" s="29" t="str"/>
+      <x:c r="B17" s="51" t="str"/>
+      <x:c r="C17" s="51" t="str"/>
+      <x:c r="D17" s="51" t="str"/>
+      <x:c r="E17" s="51" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="33" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B18" s="29" t="str"/>
-      <x:c r="C18" s="29" t="str"/>
-      <x:c r="D18" s="29" t="str"/>
-      <x:c r="E18" s="29" t="str"/>
+      <x:c r="B18" s="51" t="str"/>
+      <x:c r="C18" s="51" t="str"/>
+      <x:c r="D18" s="51" t="str"/>
+      <x:c r="E18" s="51" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="33" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B19" s="29" t="str"/>
-      <x:c r="C19" s="29" t="str"/>
-      <x:c r="D19" s="29" t="str"/>
-      <x:c r="E19" s="29" t="str"/>
+      <x:c r="B19" s="51" t="str"/>
+      <x:c r="C19" s="51" t="str"/>
+      <x:c r="D19" s="51" t="str"/>
+      <x:c r="E19" s="51" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="33" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B20" s="29" t="str"/>
-      <x:c r="C20" s="29" t="str"/>
-      <x:c r="D20" s="29" t="str"/>
-      <x:c r="E20" s="29" t="str"/>
+      <x:c r="B20" s="51" t="str"/>
+      <x:c r="C20" s="51" t="str"/>
+      <x:c r="D20" s="51" t="str"/>
+      <x:c r="E20" s="51" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="33" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B21" s="29" t="str"/>
-      <x:c r="C21" s="29" t="str"/>
-      <x:c r="D21" s="29" t="str"/>
-      <x:c r="E21" s="29" t="str"/>
+      <x:c r="B21" s="51" t="str"/>
+      <x:c r="C21" s="51" t="str"/>
+      <x:c r="D21" s="51" t="str"/>
+      <x:c r="E21" s="51" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="33" t="n">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B22" s="29" t="str"/>
-      <x:c r="C22" s="29" t="str"/>
-      <x:c r="D22" s="29" t="str"/>
-      <x:c r="E22" s="29" t="str"/>
+      <x:c r="B22" s="51" t="str"/>
+      <x:c r="C22" s="51" t="str"/>
+      <x:c r="D22" s="51" t="str"/>
+      <x:c r="E22" s="51" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="33" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B23" s="29" t="str"/>
-      <x:c r="C23" s="29" t="str"/>
-      <x:c r="D23" s="29" t="str"/>
-      <x:c r="E23" s="29" t="str"/>
+      <x:c r="B23" s="51" t="str"/>
+      <x:c r="C23" s="51" t="str"/>
+      <x:c r="D23" s="51" t="str"/>
+      <x:c r="E23" s="51" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="33" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B24" s="29" t="str"/>
-      <x:c r="C24" s="29" t="str"/>
-      <x:c r="D24" s="29" t="str"/>
-      <x:c r="E24" s="29" t="str"/>
+      <x:c r="B24" s="51" t="str"/>
+      <x:c r="C24" s="51" t="str"/>
+      <x:c r="D24" s="51" t="str"/>
+      <x:c r="E24" s="51" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="33" t="n">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B25" s="29" t="str"/>
-      <x:c r="C25" s="29" t="str"/>
-      <x:c r="D25" s="29" t="str"/>
-      <x:c r="E25" s="29" t="str"/>
+      <x:c r="B25" s="51" t="str"/>
+      <x:c r="C25" s="51" t="str"/>
+      <x:c r="D25" s="51" t="str"/>
+      <x:c r="E25" s="51" t="str"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="33" t="n">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B26" s="29" t="str"/>
-      <x:c r="C26" s="29" t="str"/>
-      <x:c r="D26" s="29" t="str"/>
-      <x:c r="E26" s="29" t="str"/>
+      <x:c r="B26" s="51" t="str"/>
+      <x:c r="C26" s="51" t="str"/>
+      <x:c r="D26" s="51" t="str"/>
+      <x:c r="E26" s="51" t="str"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="33" t="n">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B27" s="29" t="str"/>
-      <x:c r="C27" s="29" t="str"/>
-      <x:c r="D27" s="29" t="str"/>
-      <x:c r="E27" s="29" t="str"/>
+      <x:c r="B27" s="51" t="str"/>
+      <x:c r="C27" s="51" t="str"/>
+      <x:c r="D27" s="51" t="str"/>
+      <x:c r="E27" s="51" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="33" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B28" s="29" t="str"/>
-      <x:c r="C28" s="29" t="str"/>
-      <x:c r="D28" s="29" t="str"/>
-      <x:c r="E28" s="29" t="str"/>
+      <x:c r="B28" s="51" t="str"/>
+      <x:c r="C28" s="51" t="str"/>
+      <x:c r="D28" s="51" t="str"/>
+      <x:c r="E28" s="51" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="33" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="B29" s="29" t="str"/>
-      <x:c r="C29" s="29" t="str"/>
-      <x:c r="D29" s="29" t="str"/>
-      <x:c r="E29" s="29" t="str"/>
+      <x:c r="B29" s="51" t="str"/>
+      <x:c r="C29" s="51" t="str"/>
+      <x:c r="D29" s="51" t="str"/>
+      <x:c r="E29" s="51" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="33" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B30" s="29" t="str"/>
-      <x:c r="C30" s="29" t="str"/>
-      <x:c r="D30" s="29" t="str"/>
-      <x:c r="E30" s="29" t="str"/>
+      <x:c r="B30" s="51" t="str"/>
+      <x:c r="C30" s="51" t="str"/>
+      <x:c r="D30" s="51" t="str"/>
+      <x:c r="E30" s="51" t="str"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="33" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B31" s="29" t="str"/>
-      <x:c r="C31" s="29" t="str"/>
-      <x:c r="D31" s="29" t="str"/>
-      <x:c r="E31" s="29" t="str"/>
+      <x:c r="B31" s="51" t="str"/>
+      <x:c r="C31" s="51" t="str"/>
+      <x:c r="D31" s="51" t="str"/>
+      <x:c r="E31" s="51" t="str"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="33" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B32" s="29" t="str"/>
-      <x:c r="C32" s="29" t="str"/>
-      <x:c r="D32" s="29" t="str"/>
-      <x:c r="E32" s="29" t="str"/>
+      <x:c r="B32" s="51" t="str"/>
+      <x:c r="C32" s="51" t="str"/>
+      <x:c r="D32" s="51" t="str"/>
+      <x:c r="E32" s="51" t="str"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="33" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B33" s="29" t="str"/>
-      <x:c r="C33" s="29" t="str"/>
-      <x:c r="D33" s="29" t="str"/>
-      <x:c r="E33" s="29" t="str"/>
+      <x:c r="B33" s="51" t="str"/>
+      <x:c r="C33" s="51" t="str"/>
+      <x:c r="D33" s="51" t="str"/>
+      <x:c r="E33" s="51" t="str"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="33" t="n">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B34" s="29" t="str"/>
-      <x:c r="C34" s="29" t="str"/>
-      <x:c r="D34" s="29" t="str"/>
-      <x:c r="E34" s="29" t="str"/>
+      <x:c r="B34" s="51" t="str"/>
+      <x:c r="C34" s="51" t="str"/>
+      <x:c r="D34" s="51" t="str"/>
+      <x:c r="E34" s="51" t="str"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="33" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B35" s="29" t="str"/>
-      <x:c r="C35" s="29" t="str"/>
-      <x:c r="D35" s="29" t="str"/>
-      <x:c r="E35" s="29" t="str"/>
+      <x:c r="B35" s="51" t="str"/>
+      <x:c r="C35" s="51" t="str"/>
+      <x:c r="D35" s="51" t="str"/>
+      <x:c r="E35" s="51" t="str"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="33" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B36" s="29" t="str"/>
-      <x:c r="C36" s="29" t="str"/>
-      <x:c r="D36" s="29" t="str"/>
-      <x:c r="E36" s="29" t="str"/>
+      <x:c r="B36" s="51" t="str"/>
+      <x:c r="C36" s="51" t="str"/>
+      <x:c r="D36" s="51" t="str"/>
+      <x:c r="E36" s="51" t="str"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="33" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="B37" s="29" t="str"/>
-      <x:c r="C37" s="29" t="str"/>
-      <x:c r="D37" s="29" t="str"/>
-      <x:c r="E37" s="29" t="str"/>
+      <x:c r="B37" s="51" t="str"/>
+      <x:c r="C37" s="51" t="str"/>
+      <x:c r="D37" s="51" t="str"/>
+      <x:c r="E37" s="51" t="str"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="33" t="n">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="B38" s="29" t="str"/>
-      <x:c r="C38" s="29" t="str"/>
-      <x:c r="D38" s="29" t="str"/>
-      <x:c r="E38" s="29" t="str"/>
+      <x:c r="B38" s="51" t="str"/>
+      <x:c r="C38" s="51" t="str"/>
+      <x:c r="D38" s="51" t="str"/>
+      <x:c r="E38" s="51" t="str"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="33" t="n">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="B39" s="29" t="str"/>
-      <x:c r="C39" s="29" t="str"/>
-      <x:c r="D39" s="29" t="str"/>
-      <x:c r="E39" s="29" t="str"/>
+      <x:c r="B39" s="51" t="str"/>
+      <x:c r="C39" s="51" t="str"/>
+      <x:c r="D39" s="51" t="str"/>
+      <x:c r="E39" s="51" t="str"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="33" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B40" s="29" t="str"/>
-      <x:c r="C40" s="29" t="str"/>
-      <x:c r="D40" s="29" t="str"/>
-      <x:c r="E40" s="29" t="str"/>
+      <x:c r="B40" s="51" t="str"/>
+      <x:c r="C40" s="51" t="str"/>
+      <x:c r="D40" s="51" t="str"/>
+      <x:c r="E40" s="51" t="str"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="33" t="n">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="B41" s="29" t="str"/>
-      <x:c r="C41" s="29" t="str"/>
-      <x:c r="D41" s="29" t="str"/>
-      <x:c r="E41" s="29" t="str"/>
+      <x:c r="B41" s="51" t="str"/>
+      <x:c r="C41" s="51" t="str"/>
+      <x:c r="D41" s="51" t="str"/>
+      <x:c r="E41" s="51" t="str"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="33" t="n">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B42" s="29" t="str"/>
-      <x:c r="C42" s="29" t="str"/>
-      <x:c r="D42" s="29" t="str"/>
-      <x:c r="E42" s="29" t="str"/>
+      <x:c r="B42" s="51" t="str"/>
+      <x:c r="C42" s="51" t="str"/>
+      <x:c r="D42" s="51" t="str"/>
+      <x:c r="E42" s="51" t="str"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="33" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="B43" s="29" t="str"/>
-      <x:c r="C43" s="29" t="str"/>
-      <x:c r="D43" s="29" t="str"/>
-      <x:c r="E43" s="29" t="str"/>
+      <x:c r="B43" s="51" t="str"/>
+      <x:c r="C43" s="51" t="str"/>
+      <x:c r="D43" s="51" t="str"/>
+      <x:c r="E43" s="51" t="str"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="33" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="B44" s="29" t="str"/>
-      <x:c r="C44" s="29" t="str"/>
-      <x:c r="D44" s="29" t="str"/>
-      <x:c r="E44" s="29" t="str"/>
+      <x:c r="B44" s="51" t="str"/>
+      <x:c r="C44" s="51" t="str"/>
+      <x:c r="D44" s="51" t="str"/>
+      <x:c r="E44" s="51" t="str"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="33" t="n">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B45" s="29" t="str"/>
-      <x:c r="C45" s="29" t="str"/>
-      <x:c r="D45" s="29" t="str"/>
-      <x:c r="E45" s="29" t="str"/>
+      <x:c r="B45" s="51" t="str"/>
+      <x:c r="C45" s="51" t="str"/>
+      <x:c r="D45" s="51" t="str"/>
+      <x:c r="E45" s="51" t="str"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="33" t="n">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="B46" s="29" t="str"/>
-      <x:c r="C46" s="29" t="str"/>
-      <x:c r="D46" s="29" t="str"/>
-      <x:c r="E46" s="29" t="str"/>
+      <x:c r="B46" s="51" t="str"/>
+      <x:c r="C46" s="51" t="str"/>
+      <x:c r="D46" s="51" t="str"/>
+      <x:c r="E46" s="51" t="str"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="33" t="n">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="B47" s="29" t="str"/>
-      <x:c r="C47" s="29" t="str"/>
-      <x:c r="D47" s="29" t="str"/>
-      <x:c r="E47" s="29" t="str"/>
+      <x:c r="B47" s="51" t="str"/>
+      <x:c r="C47" s="51" t="str"/>
+      <x:c r="D47" s="51" t="str"/>
+      <x:c r="E47" s="51" t="str"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="33" t="n">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B48" s="29" t="str"/>
-      <x:c r="C48" s="29" t="str"/>
-      <x:c r="D48" s="29" t="str"/>
-      <x:c r="E48" s="29" t="str"/>
+      <x:c r="B48" s="51" t="str"/>
+      <x:c r="C48" s="51" t="str"/>
+      <x:c r="D48" s="51" t="str"/>
+      <x:c r="E48" s="51" t="str"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="33" t="n">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="B49" s="29" t="str"/>
-      <x:c r="C49" s="29" t="str"/>
-      <x:c r="D49" s="29" t="str"/>
-      <x:c r="E49" s="29" t="str"/>
+      <x:c r="B49" s="51" t="str"/>
+      <x:c r="C49" s="51" t="str"/>
+      <x:c r="D49" s="51" t="str"/>
+      <x:c r="E49" s="51" t="str"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="33" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B50" s="29" t="str"/>
-      <x:c r="C50" s="29" t="str"/>
-      <x:c r="D50" s="29" t="str"/>
-      <x:c r="E50" s="29" t="str"/>
+      <x:c r="B50" s="51" t="str"/>
+      <x:c r="C50" s="51" t="str"/>
+      <x:c r="D50" s="51" t="str"/>
+      <x:c r="E50" s="51" t="str"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="33" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="B51" s="29" t="str"/>
-      <x:c r="C51" s="29" t="str"/>
-      <x:c r="D51" s="29" t="str"/>
-      <x:c r="E51" s="29" t="str"/>
+      <x:c r="B51" s="51" t="str"/>
+      <x:c r="C51" s="51" t="str"/>
+      <x:c r="D51" s="51" t="str"/>
+      <x:c r="E51" s="51" t="str"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="33" t="n">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="B52" s="29" t="str"/>
-      <x:c r="C52" s="29" t="str"/>
-      <x:c r="D52" s="29" t="str"/>
-      <x:c r="E52" s="29" t="str"/>
+      <x:c r="B52" s="51" t="str"/>
+      <x:c r="C52" s="51" t="str"/>
+      <x:c r="D52" s="51" t="str"/>
+      <x:c r="E52" s="51" t="str"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="33" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="B53" s="29" t="str"/>
-      <x:c r="C53" s="29" t="str"/>
-      <x:c r="D53" s="29" t="str"/>
-      <x:c r="E53" s="29" t="str"/>
+      <x:c r="B53" s="51" t="str"/>
+      <x:c r="C53" s="51" t="str"/>
+      <x:c r="D53" s="51" t="str"/>
+      <x:c r="E53" s="51" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
     <x:mergeCell ref="A2:E2"/>
   </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="E4:E53">
+      <x:formula1>"Đang hoạt động,Ngừng hoạt động,Chờ phê duyệt"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -911,16 +930,16 @@
       <x:c r="A4" s="29" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B4" s="29" t="str">
+      <x:c r="B4" s="51" t="str">
         <x:v>BM_LT</x:v>
       </x:c>
-      <x:c r="C4" s="29" t="str">
+      <x:c r="C4" s="51" t="str">
         <x:v>Bộ môn Lập trình</x:v>
       </x:c>
-      <x:c r="D4" s="29" t="str">
+      <x:c r="D4" s="51" t="str">
         <x:v>CNTT</x:v>
       </x:c>
-      <x:c r="E4" s="29" t="str">
+      <x:c r="E4" s="51" t="str">
         <x:v>Đang hoạt động</x:v>
       </x:c>
     </x:row>
@@ -941,68 +960,124 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="36" t="str">
+      <x:c r="A1" s="48" t="str">
         <x:v>MẪU NHẬP BỘ MÔN - HƯỚNG DẪN</x:v>
       </x:c>
       <x:c r="B1" s="48"/>
       <x:c r="C1" s="36"/>
       <x:c r="D1" s="36"/>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="52"/>
+      <x:c r="B2" s="52"/>
+    </x:row>
     <x:row r="3">
-      <x:c r="A3" s="45" t="str">
+      <x:c r="A3" s="53" t="str">
         <x:v>Nội dung</x:v>
       </x:c>
-      <x:c r="B3" s="45" t="str">
+      <x:c r="B3" s="53" t="str">
         <x:v>Chi tiết</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="29" t="str">
+      <x:c r="A4" s="54" t="str">
         <x:v>Sheet nhập chính</x:v>
       </x:c>
-      <x:c r="B4" s="29" t="str">
+      <x:c r="B4" s="54" t="str">
         <x:v>Dữ liệu</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="29" t="str">
+      <x:c r="A5" s="54" t="str">
         <x:v>Dòng tiêu đề cột</x:v>
       </x:c>
-      <x:c r="B5" s="29" t="str">
+      <x:c r="B5" s="54" t="str">
         <x:v>Dòng 3</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="29" t="str">
+      <x:c r="A6" s="54" t="str">
         <x:v>Dòng bắt đầu nhập</x:v>
       </x:c>
-      <x:c r="B6" s="29" t="str">
+      <x:c r="B6" s="54" t="str">
         <x:v>Dòng 4</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="29" t="str">
+      <x:c r="A7" s="54" t="str">
         <x:v>Cột bắt buộc</x:v>
       </x:c>
-      <x:c r="B7" s="29" t="str">
+      <x:c r="B7" s="54" t="str">
         <x:v>Mã bộ môn, Tên bộ môn, Mã khoa</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="29" t="str">
+      <x:c r="A8" s="54" t="str">
         <x:v>Lưu ý</x:v>
       </x:c>
-      <x:c r="B8" s="29" t="str">
+      <x:c r="B8" s="54" t="str">
         <x:v>Mã khoa phải tồn tại trước trong hệ thống.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="29" t="str">
+      <x:c r="A9" s="54" t="str">
         <x:v>Lưu ý</x:v>
       </x:c>
-      <x:c r="B9" s="29" t="str">
+      <x:c r="B9" s="54" t="str">
         <x:v>Mã bộ môn không được trùng.</x:v>
       </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="52" t="str">
+        <x:v>Trạng thái</x:v>
+      </x:c>
+      <x:c r="B10" s="52" t="str">
+        <x:v>Đang hoạt động, Ngừng hoạt động hoặc Chờ phê duyệt.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="52" t="str">
+        <x:v>Quan trọng</x:v>
+      </x:c>
+      <x:c r="B11" s="52" t="str">
+        <x:v>Mã khoa phải là mã đang tồn tại trong hệ thống. Chỉ nhập tại sheet Dữ liệu.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="52"/>
+      <x:c r="B12" s="52"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="52"/>
+      <x:c r="B13" s="52"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="52"/>
+      <x:c r="B14" s="52"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="52"/>
+      <x:c r="B15" s="52"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="52"/>
+      <x:c r="B16" s="52"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="52"/>
+      <x:c r="B17" s="52"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="52"/>
+      <x:c r="B18" s="52"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="52"/>
+      <x:c r="B19" s="52"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="52"/>
+      <x:c r="B20" s="52"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>